<commit_message>
mmacos e5hex1_budget: regenerate e5hex1_wfe_budget.xlsx with the number formats (85900c3)
Generated by run_budget_e5hex1 at 85900c3 (its Log records the SHA).
LibreOffice-recalculated Payload WFE = 3.15580786565109 nm == coef.total
(rel 5.6e-16), shown as 3.156; PM Seg Tilt Pre WFC shown 96.792, the sigma
inputs as typed (50, 100).  Numbers unchanged from 0041307 apart from the
Monte-Carlo check column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mmacos/templates/50_sensitivities/e5hex1_budget/e5hex1_wfe_budget.xlsx
+++ b/mmacos/templates/50_sensitivities/e5hex1_budget/e5hex1_wfe_budget.xlsx
@@ -15,6 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000E+00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -52,11 +57,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1370,7 +1379,7 @@
           <t xml:space="preserve">WFE Margin</t>
         </is>
       </c>
-      <c r="K40" s="3">
+      <c r="K40" s="5">
         <f>IF(K39&gt;0,1-(K38/K39),"")</f>
       </c>
     </row>
@@ -1524,10 +1533,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <f>K4</f>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="4">
         <f>M4</f>
       </c>
       <c r="F4" t="inlineStr">
@@ -1535,10 +1544,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="4">
         <f>P4</f>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="4">
         <f>R4</f>
       </c>
       <c r="J4" t="inlineStr">
@@ -1546,7 +1555,7 @@
           <t xml:space="preserve">PM_Seg_Tilt0</t>
         </is>
       </c>
-      <c r="K4">
+      <c r="K4" s="6">
         <v>1.9358336025009344</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -1554,7 +1563,7 @@
           <t xml:space="preserve">PM_Seg_Tiltf</t>
         </is>
       </c>
-      <c r="M4">
+      <c r="M4" s="6">
         <v>1.4851440777787723e-11</v>
       </c>
       <c r="O4" t="inlineStr">
@@ -1562,7 +1571,7 @@
           <t xml:space="preserve">PM_Seg_Tilt0</t>
         </is>
       </c>
-      <c r="P4">
+      <c r="P4" s="6">
         <v>1.9358336025009344</v>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1570,10 +1579,10 @@
           <t xml:space="preserve">PM_Seg_Tiltf</t>
         </is>
       </c>
-      <c r="R4">
+      <c r="R4" s="6">
         <v>1.9358336025009344</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="7">
         <v>7.1826245980180876e-09</v>
       </c>
     </row>
@@ -1588,10 +1597,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <f>K5</f>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="4">
         <f>M5</f>
       </c>
       <c r="F5" t="inlineStr">
@@ -1599,10 +1608,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="4">
         <f>P5</f>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="4">
         <f>R5</f>
       </c>
       <c r="J5" t="inlineStr">
@@ -1610,7 +1619,7 @@
           <t xml:space="preserve">PM_Seg_Clocking0</t>
         </is>
       </c>
-      <c r="K5">
+      <c r="K5" s="6">
         <v>0.00078806646912846895</v>
       </c>
       <c r="L5" t="inlineStr">
@@ -1618,7 +1627,7 @@
           <t xml:space="preserve">PM_Seg_Clockingf</t>
         </is>
       </c>
-      <c r="M5">
+      <c r="M5" s="6">
         <v>4.8270831991257249e-15</v>
       </c>
       <c r="O5" t="inlineStr">
@@ -1626,7 +1635,7 @@
           <t xml:space="preserve">PM_Seg_Clocking0</t>
         </is>
       </c>
-      <c r="P5">
+      <c r="P5" s="6">
         <v>0.00078806646912846895</v>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1634,10 +1643,10 @@
           <t xml:space="preserve">PM_Seg_Clockingf</t>
         </is>
       </c>
-      <c r="R5">
+      <c r="R5" s="6">
         <v>0.00078806646912846895</v>
       </c>
-      <c r="T5">
+      <c r="T5" s="7">
         <v>5.155869352749949e-12</v>
       </c>
     </row>
@@ -1652,10 +1661,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="4">
         <f>K6</f>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="4">
         <f>M6</f>
       </c>
       <c r="F6" t="inlineStr">
@@ -1663,10 +1672,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="4">
         <f>P6</f>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="4">
         <f>R6</f>
       </c>
       <c r="J6" t="inlineStr">
@@ -1674,7 +1683,7 @@
           <t xml:space="preserve">PM_Seg_Decenter0</t>
         </is>
       </c>
-      <c r="K6">
+      <c r="K6" s="6">
         <v>0.037473190112308929</v>
       </c>
       <c r="L6" t="inlineStr">
@@ -1682,7 +1691,7 @@
           <t xml:space="preserve">PM_Seg_Decenterf</t>
         </is>
       </c>
-      <c r="M6">
+      <c r="M6" s="6">
         <v>2.6803267859692754e-13</v>
       </c>
       <c r="O6" t="inlineStr">
@@ -1690,7 +1699,7 @@
           <t xml:space="preserve">PM_Seg_Decenter0</t>
         </is>
       </c>
-      <c r="P6">
+      <c r="P6" s="6">
         <v>0.037473190112308929</v>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1698,10 +1707,10 @@
           <t xml:space="preserve">PM_Seg_Decenterf</t>
         </is>
       </c>
-      <c r="R6">
+      <c r="R6" s="6">
         <v>0.037473190112308929</v>
       </c>
-      <c r="T6">
+      <c r="T6" s="7">
         <v>2.7071802343592695e-10</v>
       </c>
     </row>
@@ -1716,10 +1725,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="4">
         <f>K7</f>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="4">
         <f>M7</f>
       </c>
       <c r="F7" t="inlineStr">
@@ -1727,10 +1736,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="4">
         <f>P7</f>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="4">
         <f>R7</f>
       </c>
       <c r="J7" t="inlineStr">
@@ -1738,7 +1747,7 @@
           <t xml:space="preserve">PM_Seg_Piston0</t>
         </is>
       </c>
-      <c r="K7">
+      <c r="K7" s="6">
         <v>2.5951842596076746</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -1746,7 +1755,7 @@
           <t xml:space="preserve">PM_Seg_Pistonf</t>
         </is>
       </c>
-      <c r="M7">
+      <c r="M7" s="6">
         <v>2.1936266405016069e-11</v>
       </c>
       <c r="O7" t="inlineStr">
@@ -1754,7 +1763,7 @@
           <t xml:space="preserve">PM_Seg_Piston0</t>
         </is>
       </c>
-      <c r="P7">
+      <c r="P7" s="6">
         <v>2.5951842596076746</v>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1762,10 +1771,10 @@
           <t xml:space="preserve">PM_Seg_Pistonf</t>
         </is>
       </c>
-      <c r="R7">
+      <c r="R7" s="6">
         <v>2.5951842596076746</v>
       </c>
-      <c r="T7">
+      <c r="T7" s="7">
         <v>2.5494172995042484e-08</v>
       </c>
     </row>
@@ -1780,10 +1789,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="4">
         <f>K8</f>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="4">
         <f>M8</f>
       </c>
       <c r="F8" t="inlineStr">
@@ -1791,10 +1800,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="4">
         <f>P8</f>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="4">
         <f>R8</f>
       </c>
       <c r="J8" t="inlineStr">
@@ -1802,7 +1811,7 @@
           <t xml:space="preserve">SM_Tilt0</t>
         </is>
       </c>
-      <c r="K8">
+      <c r="K8" s="6">
         <v>0.76924610705016094</v>
       </c>
       <c r="L8" t="inlineStr">
@@ -1810,7 +1819,7 @@
           <t xml:space="preserve">SM_Tiltf</t>
         </is>
       </c>
-      <c r="M8">
+      <c r="M8" s="6">
         <v>2.7606679701531778e-11</v>
       </c>
       <c r="O8" t="inlineStr">
@@ -1818,7 +1827,7 @@
           <t xml:space="preserve">SM_Tilt0</t>
         </is>
       </c>
-      <c r="P8">
+      <c r="P8" s="6">
         <v>0.76924610705016094</v>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1826,10 +1835,10 @@
           <t xml:space="preserve">SM_Tiltf</t>
         </is>
       </c>
-      <c r="R8">
+      <c r="R8" s="6">
         <v>0.76924610705016094</v>
       </c>
-      <c r="T8">
+      <c r="T8" s="7">
         <v>5.6389887805176208e-09</v>
       </c>
     </row>
@@ -1844,10 +1853,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="4">
         <f>K9</f>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="4">
         <f>M9</f>
       </c>
       <c r="F9" t="inlineStr">
@@ -1855,10 +1864,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="4">
         <f>P9</f>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="4">
         <f>R9</f>
       </c>
       <c r="J9" t="inlineStr">
@@ -1866,7 +1875,7 @@
           <t xml:space="preserve">SM_Clocking0</t>
         </is>
       </c>
-      <c r="K9">
+      <c r="K9" s="6">
         <v>0.00067921934475878879</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -1874,7 +1883,7 @@
           <t xml:space="preserve">SM_Clockingf</t>
         </is>
       </c>
-      <c r="M9">
+      <c r="M9" s="6">
         <v>1.4228959476457817e-14</v>
       </c>
       <c r="O9" t="inlineStr">
@@ -1882,7 +1891,7 @@
           <t xml:space="preserve">SM_Clocking0</t>
         </is>
       </c>
-      <c r="P9">
+      <c r="P9" s="6">
         <v>0.00067921934475878879</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1890,10 +1899,10 @@
           <t xml:space="preserve">SM_Clockingf</t>
         </is>
       </c>
-      <c r="R9">
+      <c r="R9" s="6">
         <v>0.00067921934475878879</v>
       </c>
-      <c r="T9">
+      <c r="T9" s="7">
         <v>1.2325940495195438e-11</v>
       </c>
     </row>
@@ -1908,10 +1917,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="4">
         <f>K10</f>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="4">
         <f>M10</f>
       </c>
       <c r="F10" t="inlineStr">
@@ -1919,10 +1928,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="4">
         <f>P10</f>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="4">
         <f>R10</f>
       </c>
       <c r="J10" t="inlineStr">
@@ -1930,7 +1939,7 @@
           <t xml:space="preserve">SM_Decenter0</t>
         </is>
       </c>
-      <c r="K10">
+      <c r="K10" s="6">
         <v>0.086547911717788986</v>
       </c>
       <c r="L10" t="inlineStr">
@@ -1938,7 +1947,7 @@
           <t xml:space="preserve">SM_Decenterf</t>
         </is>
       </c>
-      <c r="M10">
+      <c r="M10" s="6">
         <v>1.9263549226998585e-12</v>
       </c>
       <c r="O10" t="inlineStr">
@@ -1946,7 +1955,7 @@
           <t xml:space="preserve">SM_Decenter0</t>
         </is>
       </c>
-      <c r="P10">
+      <c r="P10" s="6">
         <v>0.086547911717788986</v>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1954,10 +1963,10 @@
           <t xml:space="preserve">SM_Decenterf</t>
         </is>
       </c>
-      <c r="R10">
+      <c r="R10" s="6">
         <v>0.086547911717788986</v>
       </c>
-      <c r="T10">
+      <c r="T10" s="7">
         <v>1.3348294662425297e-09</v>
       </c>
     </row>
@@ -1972,10 +1981,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="4">
         <f>K11</f>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="4">
         <f>M11</f>
       </c>
       <c r="F11" t="inlineStr">
@@ -1983,10 +1992,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="4">
         <f>P11</f>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="4">
         <f>R11</f>
       </c>
       <c r="J11" t="inlineStr">
@@ -1994,7 +2003,7 @@
           <t xml:space="preserve">SM_Despace0</t>
         </is>
       </c>
-      <c r="K11">
+      <c r="K11" s="6">
         <v>0.013749978844002333</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -2002,7 +2011,7 @@
           <t xml:space="preserve">SM_Despacef</t>
         </is>
       </c>
-      <c r="M11">
+      <c r="M11" s="6">
         <v>3.9205665893367622e-14</v>
       </c>
       <c r="O11" t="inlineStr">
@@ -2010,7 +2019,7 @@
           <t xml:space="preserve">SM_Despace0</t>
         </is>
       </c>
-      <c r="P11">
+      <c r="P11" s="6">
         <v>0.013749978844002333</v>
       </c>
       <c r="Q11" t="inlineStr">
@@ -2018,10 +2027,10 @@
           <t xml:space="preserve">SM_Despacef</t>
         </is>
       </c>
-      <c r="R11">
+      <c r="R11" s="6">
         <v>0.013749978844002333</v>
       </c>
-      <c r="T11">
+      <c r="T11" s="7">
         <v>5.6211829783322412e-11</v>
       </c>
     </row>
@@ -2036,10 +2045,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="4">
         <f>K12</f>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="4">
         <f>M12</f>
       </c>
       <c r="F12" t="inlineStr">
@@ -2047,10 +2056,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="4">
         <f>P12</f>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="4">
         <f>R12</f>
       </c>
       <c r="J12" t="inlineStr">
@@ -2058,7 +2067,7 @@
           <t xml:space="preserve">Lens_Tilt0</t>
         </is>
       </c>
-      <c r="K12">
+      <c r="K12" s="6">
         <v>0.0010205009952135211</v>
       </c>
       <c r="L12" t="inlineStr">
@@ -2066,7 +2075,7 @@
           <t xml:space="preserve">Lens_Tiltf</t>
         </is>
       </c>
-      <c r="M12">
+      <c r="M12" s="6">
         <v>4.0195523893540128e-06</v>
       </c>
       <c r="O12" t="inlineStr">
@@ -2074,7 +2083,7 @@
           <t xml:space="preserve">Lens_Tilt0</t>
         </is>
       </c>
-      <c r="P12">
+      <c r="P12" s="6">
         <v>0.0010205009952135211</v>
       </c>
       <c r="Q12" t="inlineStr">
@@ -2082,10 +2091,10 @@
           <t xml:space="preserve">Lens_Tiltf</t>
         </is>
       </c>
-      <c r="R12">
+      <c r="R12" s="6">
         <v>0.0010205009952135211</v>
       </c>
-      <c r="T12">
+      <c r="T12" s="7">
         <v>0.0001976300288636717</v>
       </c>
     </row>
@@ -2100,10 +2109,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="4">
         <f>K13</f>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="4">
         <f>M13</f>
       </c>
       <c r="F13" t="inlineStr">
@@ -2111,10 +2120,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="4">
         <f>P13</f>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="4">
         <f>R13</f>
       </c>
       <c r="J13" t="inlineStr">
@@ -2122,7 +2131,7 @@
           <t xml:space="preserve">Lens_Clocking0</t>
         </is>
       </c>
-      <c r="K13">
+      <c r="K13" s="6">
         <v>2.7430228103053335e-05</v>
       </c>
       <c r="L13" t="inlineStr">
@@ -2130,7 +2139,7 @@
           <t xml:space="preserve">Lens_Clockingf</t>
         </is>
       </c>
-      <c r="M13">
+      <c r="M13" s="6">
         <v>6.7753608588838605e-07</v>
       </c>
       <c r="O13" t="inlineStr">
@@ -2138,7 +2147,7 @@
           <t xml:space="preserve">Lens_Clocking0</t>
         </is>
       </c>
-      <c r="P13">
+      <c r="P13" s="6">
         <v>2.7430228103053335e-05</v>
       </c>
       <c r="Q13" t="inlineStr">
@@ -2146,10 +2155,10 @@
           <t xml:space="preserve">Lens_Clockingf</t>
         </is>
       </c>
-      <c r="R13">
+      <c r="R13" s="6">
         <v>2.7430228103053335e-05</v>
       </c>
-      <c r="T13">
+      <c r="T13" s="7">
         <v>6.8980623528901831e-05</v>
       </c>
     </row>
@@ -2164,10 +2173,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="4">
         <f>K14</f>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="4">
         <f>M14</f>
       </c>
       <c r="F14" t="inlineStr">
@@ -2175,10 +2184,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="4">
         <f>P14</f>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="4">
         <f>R14</f>
       </c>
       <c r="J14" t="inlineStr">
@@ -2186,7 +2195,7 @@
           <t xml:space="preserve">Lens_Decenter0</t>
         </is>
       </c>
-      <c r="K14">
+      <c r="K14" s="6">
         <v>0.00065468793000924706</v>
       </c>
       <c r="L14" t="inlineStr">
@@ -2194,7 +2203,7 @@
           <t xml:space="preserve">Lens_Decenterf</t>
         </is>
       </c>
-      <c r="M14">
+      <c r="M14" s="6">
         <v>1.9259726381598439e-06</v>
       </c>
       <c r="O14" t="inlineStr">
@@ -2202,7 +2211,7 @@
           <t xml:space="preserve">Lens_Decenter0</t>
         </is>
       </c>
-      <c r="P14">
+      <c r="P14" s="6">
         <v>0.00065468793000924706</v>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2210,10 +2219,10 @@
           <t xml:space="preserve">Lens_Decenterf</t>
         </is>
       </c>
-      <c r="R14">
+      <c r="R14" s="6">
         <v>0.00065468793000924706</v>
       </c>
-      <c r="T14">
+      <c r="T14" s="7">
         <v>0.0001946825965501424</v>
       </c>
     </row>
@@ -2228,10 +2237,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="4">
         <f>K15</f>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="4">
         <f>M15</f>
       </c>
       <c r="F15" t="inlineStr">
@@ -2239,10 +2248,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="4">
         <f>P15</f>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="4">
         <f>R15</f>
       </c>
       <c r="J15" t="inlineStr">
@@ -2250,7 +2259,7 @@
           <t xml:space="preserve">Lens_Despace0</t>
         </is>
       </c>
-      <c r="K15">
+      <c r="K15" s="6">
         <v>0.00019826794169779813</v>
       </c>
       <c r="L15" t="inlineStr">
@@ -2258,7 +2267,7 @@
           <t xml:space="preserve">Lens_Despacef</t>
         </is>
       </c>
-      <c r="M15">
+      <c r="M15" s="6">
         <v>1.3092191012421147e-05</v>
       </c>
       <c r="O15" t="inlineStr">
@@ -2266,7 +2275,7 @@
           <t xml:space="preserve">Lens_Despace0</t>
         </is>
       </c>
-      <c r="P15">
+      <c r="P15" s="6">
         <v>0.00019826794169779813</v>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2274,10 +2283,10 @@
           <t xml:space="preserve">Lens_Despacef</t>
         </is>
       </c>
-      <c r="R15">
+      <c r="R15" s="6">
         <v>0.00019826794169779813</v>
       </c>
-      <c r="T15">
+      <c r="T15" s="7">
         <v>0.0015302912020565033</v>
       </c>
     </row>
@@ -2292,10 +2301,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="4">
         <f>K16</f>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="4">
         <f>M16</f>
       </c>
       <c r="F16" t="inlineStr">
@@ -2303,10 +2312,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="4">
         <f>P16</f>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="4">
         <f>R16</f>
       </c>
       <c r="J16" t="inlineStr">
@@ -2314,7 +2323,7 @@
           <t xml:space="preserve">FPA_Tilt0</t>
         </is>
       </c>
-      <c r="K16">
+      <c r="K16" s="6">
         <v>8.7212433861463843e-06</v>
       </c>
       <c r="L16" t="inlineStr">
@@ -2322,7 +2331,7 @@
           <t xml:space="preserve">FPA_Tiltf</t>
         </is>
       </c>
-      <c r="M16">
+      <c r="M16" s="6">
         <v>4.7708084966316727e-06</v>
       </c>
       <c r="O16" t="inlineStr">
@@ -2330,7 +2339,7 @@
           <t xml:space="preserve">FPA_Tilt0</t>
         </is>
       </c>
-      <c r="P16">
+      <c r="P16" s="6">
         <v>8.7212433861463843e-06</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2338,10 +2347,10 @@
           <t xml:space="preserve">FPA_Tiltf</t>
         </is>
       </c>
-      <c r="R16">
+      <c r="R16" s="6">
         <v>8.7212433861463843e-06</v>
       </c>
-      <c r="T16">
+      <c r="T16" s="7">
         <v>0.00023678390616811742</v>
       </c>
     </row>
@@ -2356,10 +2365,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="4">
         <f>K17</f>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="4">
         <f>M17</f>
       </c>
       <c r="F17" t="inlineStr">
@@ -2367,10 +2376,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="4">
         <f>P17</f>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="4">
         <f>R17</f>
       </c>
       <c r="J17" t="inlineStr">
@@ -2378,7 +2387,7 @@
           <t xml:space="preserve">FPA_Clocking0</t>
         </is>
       </c>
-      <c r="K17">
+      <c r="K17" s="6">
         <v>0.00023710885550309703</v>
       </c>
       <c r="L17" t="inlineStr">
@@ -2386,7 +2395,7 @@
           <t xml:space="preserve">FPA_Clockingf</t>
         </is>
       </c>
-      <c r="M17">
+      <c r="M17" s="6">
         <v>0.00012292676145291275</v>
       </c>
       <c r="O17" t="inlineStr">
@@ -2394,7 +2403,7 @@
           <t xml:space="preserve">FPA_Clocking0</t>
         </is>
       </c>
-      <c r="P17">
+      <c r="P17" s="6">
         <v>0.00023710885550309703</v>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2402,10 +2411,10 @@
           <t xml:space="preserve">FPA_Clockingf</t>
         </is>
       </c>
-      <c r="R17">
+      <c r="R17" s="6">
         <v>0.00023710885550309703</v>
       </c>
-      <c r="T17">
+      <c r="T17" s="7">
         <v>0.012945600856296155</v>
       </c>
     </row>
@@ -2420,10 +2429,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="4">
         <f>K18</f>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="4">
         <f>M18</f>
       </c>
       <c r="F18" t="inlineStr">
@@ -2431,10 +2440,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="4">
         <f>P18</f>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="4">
         <f>R18</f>
       </c>
       <c r="J18" t="inlineStr">
@@ -2442,7 +2451,7 @@
           <t xml:space="preserve">FPA_Decenter0</t>
         </is>
       </c>
-      <c r="K18">
+      <c r="K18" s="6">
         <v>0.014843655321773159</v>
       </c>
       <c r="L18" t="inlineStr">
@@ -2450,7 +2459,7 @@
           <t xml:space="preserve">FPA_Decenterf</t>
         </is>
       </c>
-      <c r="M18">
+      <c r="M18" s="6">
         <v>2.0396876242563919e-06</v>
       </c>
       <c r="O18" t="inlineStr">
@@ -2458,7 +2467,7 @@
           <t xml:space="preserve">FPA_Decenter0</t>
         </is>
       </c>
-      <c r="P18">
+      <c r="P18" s="6">
         <v>0.014843655321773159</v>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2466,10 +2475,10 @@
           <t xml:space="preserve">FPA_Decenterf</t>
         </is>
       </c>
-      <c r="R18">
+      <c r="R18" s="6">
         <v>0.014843655321773159</v>
       </c>
-      <c r="T18">
+      <c r="T18" s="7">
         <v>0.00020281322302222442</v>
       </c>
     </row>
@@ -2484,10 +2493,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="4">
         <f>K19</f>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="4">
         <f>M19</f>
       </c>
       <c r="F19" t="inlineStr">
@@ -2495,10 +2504,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="4">
         <f>P19</f>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="4">
         <f>R19</f>
       </c>
       <c r="J19" t="inlineStr">
@@ -2506,7 +2515,7 @@
           <t xml:space="preserve">FPA_Despace0</t>
         </is>
       </c>
-      <c r="K19">
+      <c r="K19" s="6">
         <v>0.00012872483937956432</v>
       </c>
       <c r="L19" t="inlineStr">
@@ -2514,7 +2523,7 @@
           <t xml:space="preserve">FPA_Despacef</t>
         </is>
       </c>
-      <c r="M19">
+      <c r="M19" s="6">
         <v>3.0925496477753998e-07</v>
       </c>
       <c r="O19" t="inlineStr">
@@ -2522,7 +2531,7 @@
           <t xml:space="preserve">FPA_Despace0</t>
         </is>
       </c>
-      <c r="P19">
+      <c r="P19" s="6">
         <v>0.00012872483937956432</v>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2530,10 +2539,10 @@
           <t xml:space="preserve">FPA_Despacef</t>
         </is>
       </c>
-      <c r="R19">
+      <c r="R19" s="6">
         <v>0.00012872483937956432</v>
       </c>
-      <c r="T19">
+      <c r="T19" s="7">
         <v>3.5681533689641626e-05</v>
       </c>
     </row>
@@ -2548,10 +2557,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="4">
         <f>K20</f>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="4">
         <f>M20</f>
       </c>
       <c r="F20" t="inlineStr">
@@ -2559,10 +2568,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="4">
         <f>P20</f>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="4">
         <f>R20</f>
       </c>
       <c r="J20" t="inlineStr">
@@ -2570,7 +2579,7 @@
           <t xml:space="preserve">WFS_Sensing_Error0</t>
         </is>
       </c>
-      <c r="K20">
+      <c r="K20" s="6">
         <v>0</v>
       </c>
       <c r="L20" t="inlineStr">
@@ -2578,7 +2587,7 @@
           <t xml:space="preserve">WFS_Sensing_Errorf</t>
         </is>
       </c>
-      <c r="M20">
+      <c r="M20" s="6">
         <v>0.030611412363172892</v>
       </c>
       <c r="O20" t="inlineStr">
@@ -2586,7 +2595,7 @@
           <t xml:space="preserve">WFS_Sensing_Error0</t>
         </is>
       </c>
-      <c r="P20">
+      <c r="P20" s="6">
         <v>0</v>
       </c>
       <c r="Q20" t="inlineStr">
@@ -2594,10 +2603,10 @@
           <t xml:space="preserve">WFS_Sensing_Errorf</t>
         </is>
       </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="T20">
+      <c r="R20" s="6">
+        <v>0</v>
+      </c>
+      <c r="T20" s="7">
         <v>0.091706500572057009</v>
       </c>
     </row>
@@ -2612,10 +2621,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="4">
         <f>K21</f>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="4">
         <f>M21</f>
       </c>
       <c r="F21" t="inlineStr">
@@ -2623,10 +2632,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="4">
         <f>P21</f>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="4">
         <f>R21</f>
       </c>
       <c r="J21" t="inlineStr">
@@ -2634,7 +2643,7 @@
           <t xml:space="preserve">PM_Seg_Tilt_Actuator0</t>
         </is>
       </c>
-      <c r="K21">
+      <c r="K21" s="6">
         <v>0</v>
       </c>
       <c r="L21" t="inlineStr">
@@ -2642,7 +2651,7 @@
           <t xml:space="preserve">PM_Seg_Tilt_Actuatorf</t>
         </is>
       </c>
-      <c r="M21">
+      <c r="M21" s="6">
         <v>1.9358336025009344</v>
       </c>
       <c r="O21" t="inlineStr">
@@ -2650,7 +2659,7 @@
           <t xml:space="preserve">PM_Seg_Tilt_Actuator0</t>
         </is>
       </c>
-      <c r="P21">
+      <c r="P21" s="6">
         <v>0</v>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2658,10 +2667,10 @@
           <t xml:space="preserve">PM_Seg_Tilt_Actuatorf</t>
         </is>
       </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
-      <c r="T21">
+      <c r="R21" s="6">
+        <v>0</v>
+      </c>
+      <c r="T21" s="7">
         <v>1.290981619687563</v>
       </c>
     </row>
@@ -2676,10 +2685,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="4">
         <f>K22</f>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="4">
         <f>M22</f>
       </c>
       <c r="F22" t="inlineStr">
@@ -2687,10 +2696,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="4">
         <f>P22</f>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="4">
         <f>R22</f>
       </c>
       <c r="J22" t="inlineStr">
@@ -2698,7 +2707,7 @@
           <t xml:space="preserve">PM_Seg_Clocking_Actuator0</t>
         </is>
       </c>
-      <c r="K22">
+      <c r="K22" s="6">
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr">
@@ -2706,7 +2715,7 @@
           <t xml:space="preserve">PM_Seg_Clocking_Actuatorf</t>
         </is>
       </c>
-      <c r="M22">
+      <c r="M22" s="6">
         <v>0.00078806646912846895</v>
       </c>
       <c r="O22" t="inlineStr">
@@ -2714,7 +2723,7 @@
           <t xml:space="preserve">PM_Seg_Clocking_Actuator0</t>
         </is>
       </c>
-      <c r="P22">
+      <c r="P22" s="6">
         <v>0</v>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2722,10 +2731,10 @@
           <t xml:space="preserve">PM_Seg_Clocking_Actuatorf</t>
         </is>
       </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
-      <c r="T22">
+      <c r="R22" s="6">
+        <v>0</v>
+      </c>
+      <c r="T22" s="7">
         <v>0.00052109120833285954</v>
       </c>
     </row>
@@ -2740,10 +2749,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="4">
         <f>K23</f>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="4">
         <f>M23</f>
       </c>
       <c r="F23" t="inlineStr">
@@ -2751,10 +2760,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="4">
         <f>P23</f>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="4">
         <f>R23</f>
       </c>
       <c r="J23" t="inlineStr">
@@ -2762,7 +2771,7 @@
           <t xml:space="preserve">PM_Seg_Decenter_Actuator0</t>
         </is>
       </c>
-      <c r="K23">
+      <c r="K23" s="6">
         <v>0</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -2770,7 +2779,7 @@
           <t xml:space="preserve">PM_Seg_Decenter_Actuatorf</t>
         </is>
       </c>
-      <c r="M23">
+      <c r="M23" s="6">
         <v>0.037473190112308929</v>
       </c>
       <c r="O23" t="inlineStr">
@@ -2778,7 +2787,7 @@
           <t xml:space="preserve">PM_Seg_Decenter_Actuator0</t>
         </is>
       </c>
-      <c r="P23">
+      <c r="P23" s="6">
         <v>0</v>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2786,10 +2795,10 @@
           <t xml:space="preserve">PM_Seg_Decenter_Actuatorf</t>
         </is>
       </c>
-      <c r="R23">
-        <v>0</v>
-      </c>
-      <c r="T23">
+      <c r="R23" s="6">
+        <v>0</v>
+      </c>
+      <c r="T23" s="7">
         <v>0.037507160302343925</v>
       </c>
     </row>
@@ -2804,10 +2813,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="4">
         <f>K24</f>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="4">
         <f>M24</f>
       </c>
       <c r="F24" t="inlineStr">
@@ -2815,10 +2824,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G24" s="2">
+      <c r="G24" s="4">
         <f>P24</f>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="4">
         <f>R24</f>
       </c>
       <c r="J24" t="inlineStr">
@@ -2826,7 +2835,7 @@
           <t xml:space="preserve">PM_Seg_Piston_Actuator0</t>
         </is>
       </c>
-      <c r="K24">
+      <c r="K24" s="6">
         <v>0</v>
       </c>
       <c r="L24" t="inlineStr">
@@ -2834,7 +2843,7 @@
           <t xml:space="preserve">PM_Seg_Piston_Actuatorf</t>
         </is>
       </c>
-      <c r="M24">
+      <c r="M24" s="6">
         <v>2.5951842596076746</v>
       </c>
       <c r="O24" t="inlineStr">
@@ -2842,7 +2851,7 @@
           <t xml:space="preserve">PM_Seg_Piston_Actuator0</t>
         </is>
       </c>
-      <c r="P24">
+      <c r="P24" s="6">
         <v>0</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2850,10 +2859,10 @@
           <t xml:space="preserve">PM_Seg_Piston_Actuatorf</t>
         </is>
       </c>
-      <c r="R24">
-        <v>0</v>
-      </c>
-      <c r="T24">
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="T24" s="7">
         <v>2.6230583308107964</v>
       </c>
     </row>
@@ -2868,10 +2877,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="4">
         <f>K25</f>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="4">
         <f>M25</f>
       </c>
       <c r="F25" t="inlineStr">
@@ -2879,10 +2888,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G25" s="2">
+      <c r="G25" s="4">
         <f>P25</f>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="4">
         <f>R25</f>
       </c>
       <c r="J25" t="inlineStr">
@@ -2890,7 +2899,7 @@
           <t xml:space="preserve">SM_Tilt_Actuator0</t>
         </is>
       </c>
-      <c r="K25">
+      <c r="K25" s="6">
         <v>0</v>
       </c>
       <c r="L25" t="inlineStr">
@@ -2898,7 +2907,7 @@
           <t xml:space="preserve">SM_Tilt_Actuatorf</t>
         </is>
       </c>
-      <c r="M25">
+      <c r="M25" s="6">
         <v>0.76924610705016094</v>
       </c>
       <c r="O25" t="inlineStr">
@@ -2906,7 +2915,7 @@
           <t xml:space="preserve">SM_Tilt_Actuator0</t>
         </is>
       </c>
-      <c r="P25">
+      <c r="P25" s="6">
         <v>0</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2914,10 +2923,10 @@
           <t xml:space="preserve">SM_Tilt_Actuatorf</t>
         </is>
       </c>
-      <c r="R25">
-        <v>0</v>
-      </c>
-      <c r="T25">
+      <c r="R25" s="6">
+        <v>0</v>
+      </c>
+      <c r="T25" s="7">
         <v>1.2136165690914535</v>
       </c>
     </row>
@@ -2932,10 +2941,10 @@
           <t xml:space="preserve">nrad</t>
         </is>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="4">
         <f>K26</f>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="4">
         <f>M26</f>
       </c>
       <c r="F26" t="inlineStr">
@@ -2943,10 +2952,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G26" s="2">
+      <c r="G26" s="4">
         <f>P26</f>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="4">
         <f>R26</f>
       </c>
       <c r="J26" t="inlineStr">
@@ -2954,7 +2963,7 @@
           <t xml:space="preserve">SM_Clocking_Actuator0</t>
         </is>
       </c>
-      <c r="K26">
+      <c r="K26" s="6">
         <v>0</v>
       </c>
       <c r="L26" t="inlineStr">
@@ -2962,7 +2971,7 @@
           <t xml:space="preserve">SM_Clocking_Actuatorf</t>
         </is>
       </c>
-      <c r="M26">
+      <c r="M26" s="6">
         <v>0.00067921934475878879</v>
       </c>
       <c r="O26" t="inlineStr">
@@ -2970,7 +2979,7 @@
           <t xml:space="preserve">SM_Clocking_Actuator0</t>
         </is>
       </c>
-      <c r="P26">
+      <c r="P26" s="6">
         <v>0</v>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2978,10 +2987,10 @@
           <t xml:space="preserve">SM_Clocking_Actuatorf</t>
         </is>
       </c>
-      <c r="R26">
-        <v>0</v>
-      </c>
-      <c r="T26">
+      <c r="R26" s="6">
+        <v>0</v>
+      </c>
+      <c r="T26" s="7">
         <v>0.0011046390626261334</v>
       </c>
     </row>
@@ -2996,10 +3005,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="4">
         <f>K27</f>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="4">
         <f>M27</f>
       </c>
       <c r="F27" t="inlineStr">
@@ -3007,10 +3016,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G27" s="2">
+      <c r="G27" s="4">
         <f>P27</f>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="4">
         <f>R27</f>
       </c>
       <c r="J27" t="inlineStr">
@@ -3018,7 +3027,7 @@
           <t xml:space="preserve">SM_Decenter_Actuator0</t>
         </is>
       </c>
-      <c r="K27">
+      <c r="K27" s="6">
         <v>0</v>
       </c>
       <c r="L27" t="inlineStr">
@@ -3026,7 +3035,7 @@
           <t xml:space="preserve">SM_Decenter_Actuatorf</t>
         </is>
       </c>
-      <c r="M27">
+      <c r="M27" s="6">
         <v>0.086547911717788986</v>
       </c>
       <c r="O27" t="inlineStr">
@@ -3034,7 +3043,7 @@
           <t xml:space="preserve">SM_Decenter_Actuator0</t>
         </is>
       </c>
-      <c r="P27">
+      <c r="P27" s="6">
         <v>0</v>
       </c>
       <c r="Q27" t="inlineStr">
@@ -3042,10 +3051,10 @@
           <t xml:space="preserve">SM_Decenter_Actuatorf</t>
         </is>
       </c>
-      <c r="R27">
-        <v>0</v>
-      </c>
-      <c r="T27">
+      <c r="R27" s="6">
+        <v>0</v>
+      </c>
+      <c r="T27" s="7">
         <v>0.086372490811694735</v>
       </c>
     </row>
@@ -3060,10 +3069,10 @@
           <t xml:space="preserve">nm</t>
         </is>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="4">
         <f>K28</f>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="4">
         <f>M28</f>
       </c>
       <c r="F28" t="inlineStr">
@@ -3071,10 +3080,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G28" s="2">
+      <c r="G28" s="4">
         <f>P28</f>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="4">
         <f>R28</f>
       </c>
       <c r="J28" t="inlineStr">
@@ -3082,7 +3091,7 @@
           <t xml:space="preserve">SM_Despace_Actuator0</t>
         </is>
       </c>
-      <c r="K28">
+      <c r="K28" s="6">
         <v>0</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -3090,7 +3099,7 @@
           <t xml:space="preserve">SM_Despace_Actuatorf</t>
         </is>
       </c>
-      <c r="M28">
+      <c r="M28" s="6">
         <v>0.013749978844002333</v>
       </c>
       <c r="O28" t="inlineStr">
@@ -3098,7 +3107,7 @@
           <t xml:space="preserve">SM_Despace_Actuator0</t>
         </is>
       </c>
-      <c r="P28">
+      <c r="P28" s="6">
         <v>0</v>
       </c>
       <c r="Q28" t="inlineStr">
@@ -3106,10 +3115,10 @@
           <t xml:space="preserve">SM_Despace_Actuatorf</t>
         </is>
       </c>
-      <c r="R28">
-        <v>0</v>
-      </c>
-      <c r="T28">
+      <c r="R28" s="6">
+        <v>0</v>
+      </c>
+      <c r="T28" s="7">
         <v>0.013777245744835839</v>
       </c>
     </row>
@@ -3410,7 +3419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">generated 2026-10-16 09:13:41 by macos.budget.write_workbook</t>
+          <t xml:space="preserve">generated 2026-10-16 09:33:05 by macos.budget.write_workbook</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3475,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACOS_resources 64769ae</t>
+          <t xml:space="preserve">MACOS_resources 85900c3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
mmacos e5hex1_budget: regenerate e5hex1_wfe_budget.xlsx with the input formats and the legend (1d10ab5)
Generated by run_budget_e5hex1 at 1d10ab5 (its Log records the SHA).
LibreOffice-recalculated Payload WFE = 3.15580786565109 nm == coef.total
(rel 5.6e-16), shown 3.156.  Inputs now read three decimals: PM Seg Piston
sigma shown 115.470 (stored 115.470053837925), PM Seg Tilt 50.000.  WFE!M1
carries the white = input / gray = formula legend.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mmacos/templates/50_sensitivities/e5hex1_budget/e5hex1_wfe_budget.xlsx
+++ b/mmacos/templates/50_sensitivities/e5hex1_budget/e5hex1_wfe_budget.xlsx
@@ -113,6 +113,11 @@
           <t xml:space="preserve">Total WFE</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">white cells = inputs you edit; gray cells = formulas (computed)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -204,7 +209,7 @@
           <t xml:space="preserve">PM Seg Tilt</t>
         </is>
       </c>
-      <c r="C4">
+      <c r="C4" s="7">
         <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -218,7 +223,7 @@
       <c r="F4" s="2">
         <f>C4*Coefficients!E4</f>
       </c>
-      <c r="G4">
+      <c r="G4" s="7">
         <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -242,7 +247,7 @@
           <t xml:space="preserve">PM Seg Clocking</t>
         </is>
       </c>
-      <c r="C5">
+      <c r="C5" s="7">
         <v>100</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -256,7 +261,7 @@
       <c r="F5" s="2">
         <f>C5*Coefficients!E5</f>
       </c>
-      <c r="G5">
+      <c r="G5" s="7">
         <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -280,7 +285,7 @@
           <t xml:space="preserve">PM Seg Decenter</t>
         </is>
       </c>
-      <c r="C6">
+      <c r="C6" s="7">
         <v>100</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -294,7 +299,7 @@
       <c r="F6" s="2">
         <f>C6*Coefficients!E6</f>
       </c>
-      <c r="G6">
+      <c r="G6" s="7">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -318,7 +323,7 @@
           <t xml:space="preserve">PM Seg Piston</t>
         </is>
       </c>
-      <c r="C7">
+      <c r="C7" s="7">
         <v>115.47005383792516</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -332,7 +337,7 @@
       <c r="F7" s="2">
         <f>C7*Coefficients!E7</f>
       </c>
-      <c r="G7">
+      <c r="G7" s="7">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
@@ -361,7 +366,7 @@
           <t xml:space="preserve">SM Tilt</t>
         </is>
       </c>
-      <c r="C8">
+      <c r="C8" s="7">
         <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -375,7 +380,7 @@
       <c r="F8" s="2">
         <f>C8*Coefficients!E8</f>
       </c>
-      <c r="G8">
+      <c r="G8" s="7">
         <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
@@ -399,7 +404,7 @@
           <t xml:space="preserve">SM Clocking</t>
         </is>
       </c>
-      <c r="C9">
+      <c r="C9" s="7">
         <v>100</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -413,7 +418,7 @@
       <c r="F9" s="2">
         <f>C9*Coefficients!E9</f>
       </c>
-      <c r="G9">
+      <c r="G9" s="7">
         <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
@@ -437,7 +442,7 @@
           <t xml:space="preserve">SM Decenter</t>
         </is>
       </c>
-      <c r="C10">
+      <c r="C10" s="7">
         <v>100</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -451,7 +456,7 @@
       <c r="F10" s="2">
         <f>C10*Coefficients!E10</f>
       </c>
-      <c r="G10">
+      <c r="G10" s="7">
         <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
@@ -475,7 +480,7 @@
           <t xml:space="preserve">SM Despace</t>
         </is>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>115.47005383792516</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -489,7 +494,7 @@
       <c r="F11" s="2">
         <f>C11*Coefficients!E11</f>
       </c>
-      <c r="G11">
+      <c r="G11" s="7">
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr">
@@ -518,7 +523,7 @@
           <t xml:space="preserve">Lens Tilt</t>
         </is>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>50</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -532,7 +537,7 @@
       <c r="F12" s="2">
         <f>C12*Coefficients!E12</f>
       </c>
-      <c r="G12">
+      <c r="G12" s="7">
         <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
@@ -556,7 +561,7 @@
           <t xml:space="preserve">Lens Clocking</t>
         </is>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>100</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -570,7 +575,7 @@
       <c r="F13" s="2">
         <f>C13*Coefficients!E13</f>
       </c>
-      <c r="G13">
+      <c r="G13" s="7">
         <v>0</v>
       </c>
       <c r="H13" t="inlineStr">
@@ -594,7 +599,7 @@
           <t xml:space="preserve">Lens Decenter</t>
         </is>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>100</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -608,7 +613,7 @@
       <c r="F14" s="2">
         <f>C14*Coefficients!E14</f>
       </c>
-      <c r="G14">
+      <c r="G14" s="7">
         <v>0</v>
       </c>
       <c r="H14" t="inlineStr">
@@ -632,7 +637,7 @@
           <t xml:space="preserve">Lens Despace</t>
         </is>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>115.47005383792516</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -646,7 +651,7 @@
       <c r="F15" s="2">
         <f>C15*Coefficients!E15</f>
       </c>
-      <c r="G15">
+      <c r="G15" s="7">
         <v>0</v>
       </c>
       <c r="H15" t="inlineStr">
@@ -675,7 +680,7 @@
           <t xml:space="preserve">FPA Tilt</t>
         </is>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>50</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -689,7 +694,7 @@
       <c r="F16" s="2">
         <f>C16*Coefficients!E16</f>
       </c>
-      <c r="G16">
+      <c r="G16" s="7">
         <v>0</v>
       </c>
       <c r="H16" t="inlineStr">
@@ -713,7 +718,7 @@
           <t xml:space="preserve">FPA Clocking</t>
         </is>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>100</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -727,7 +732,7 @@
       <c r="F17" s="2">
         <f>C17*Coefficients!E17</f>
       </c>
-      <c r="G17">
+      <c r="G17" s="7">
         <v>0</v>
       </c>
       <c r="H17" t="inlineStr">
@@ -751,7 +756,7 @@
           <t xml:space="preserve">FPA Decenter</t>
         </is>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>100</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -765,7 +770,7 @@
       <c r="F18" s="2">
         <f>C18*Coefficients!E18</f>
       </c>
-      <c r="G18">
+      <c r="G18" s="7">
         <v>0</v>
       </c>
       <c r="H18" t="inlineStr">
@@ -789,7 +794,7 @@
           <t xml:space="preserve">FPA Despace</t>
         </is>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>115.47005383792516</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -803,7 +808,7 @@
       <c r="F19" s="2">
         <f>C19*Coefficients!E19</f>
       </c>
-      <c r="G19">
+      <c r="G19" s="7">
         <v>0</v>
       </c>
       <c r="H19" t="inlineStr">
@@ -832,7 +837,7 @@
           <t xml:space="preserve">WFS Sensing Error</t>
         </is>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>3</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -846,7 +851,7 @@
       <c r="F20" s="2">
         <f>C20*Coefficients!E20</f>
       </c>
-      <c r="G20">
+      <c r="G20" s="7">
         <v>0</v>
       </c>
       <c r="H20" t="inlineStr">
@@ -870,7 +875,7 @@
           <t xml:space="preserve">PM Seg Tilt Actuator</t>
         </is>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>0.66193024493078101</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -884,7 +889,7 @@
       <c r="F21" s="2">
         <f>C21*Coefficients!E21</f>
       </c>
-      <c r="G21">
+      <c r="G21" s="7">
         <v>0</v>
       </c>
       <c r="H21" t="inlineStr">
@@ -908,7 +913,7 @@
           <t xml:space="preserve">PM Seg Clocking Actuator</t>
         </is>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>0.66193024493078101</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -922,7 +927,7 @@
       <c r="F22" s="2">
         <f>C22*Coefficients!E22</f>
       </c>
-      <c r="G22">
+      <c r="G22" s="7">
         <v>0</v>
       </c>
       <c r="H22" t="inlineStr">
@@ -946,7 +951,7 @@
           <t xml:space="preserve">PM Seg Decenter Actuator</t>
         </is>
       </c>
-      <c r="C23">
+      <c r="C23" s="7">
         <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -960,7 +965,7 @@
       <c r="F23" s="2">
         <f>C23*Coefficients!E23</f>
       </c>
-      <c r="G23">
+      <c r="G23" s="7">
         <v>0</v>
       </c>
       <c r="H23" t="inlineStr">
@@ -984,7 +989,7 @@
           <t xml:space="preserve">PM Seg Piston Actuator</t>
         </is>
       </c>
-      <c r="C24">
+      <c r="C24" s="7">
         <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -998,7 +1003,7 @@
       <c r="F24" s="2">
         <f>C24*Coefficients!E24</f>
       </c>
-      <c r="G24">
+      <c r="G24" s="7">
         <v>0</v>
       </c>
       <c r="H24" t="inlineStr">
@@ -1022,7 +1027,7 @@
           <t xml:space="preserve">SM Tilt Actuator</t>
         </is>
       </c>
-      <c r="C25">
+      <c r="C25" s="7">
         <v>1.6260162601626018</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -1036,7 +1041,7 @@
       <c r="F25" s="2">
         <f>C25*Coefficients!E25</f>
       </c>
-      <c r="G25">
+      <c r="G25" s="7">
         <v>0</v>
       </c>
       <c r="H25" t="inlineStr">
@@ -1060,7 +1065,7 @@
           <t xml:space="preserve">SM Clocking Actuator</t>
         </is>
       </c>
-      <c r="C26">
+      <c r="C26" s="7">
         <v>1.6260162601626018</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1074,7 +1079,7 @@
       <c r="F26" s="2">
         <f>C26*Coefficients!E26</f>
       </c>
-      <c r="G26">
+      <c r="G26" s="7">
         <v>0</v>
       </c>
       <c r="H26" t="inlineStr">
@@ -1098,7 +1103,7 @@
           <t xml:space="preserve">SM Decenter Actuator</t>
         </is>
       </c>
-      <c r="C27">
+      <c r="C27" s="7">
         <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -1112,7 +1117,7 @@
       <c r="F27" s="2">
         <f>C27*Coefficients!E27</f>
       </c>
-      <c r="G27">
+      <c r="G27" s="7">
         <v>0</v>
       </c>
       <c r="H27" t="inlineStr">
@@ -1136,7 +1141,7 @@
           <t xml:space="preserve">SM Despace Actuator</t>
         </is>
       </c>
-      <c r="C28">
+      <c r="C28" s="7">
         <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -1150,7 +1155,7 @@
       <c r="F28" s="2">
         <f>C28*Coefficients!E28</f>
       </c>
-      <c r="G28">
+      <c r="G28" s="7">
         <v>0</v>
       </c>
       <c r="H28" t="inlineStr">
@@ -1333,7 +1338,7 @@
           <t xml:space="preserve">Design WFE</t>
         </is>
       </c>
-      <c r="C37">
+      <c r="C37" s="7">
         <v>0</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -3419,7 +3424,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">generated 2026-10-16 09:33:05 by macos.budget.write_workbook</t>
+          <t xml:space="preserve">generated 2026-10-16 10:23:45 by macos.budget.write_workbook</t>
         </is>
       </c>
     </row>
@@ -3454,28 +3459,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFS: "WFS Sensing Error" (WFE row 20) sigma 3 nm is WHITE per-sample noise (Redding 2014 Eq. 32, the default ruled 2026-10-16): post-WFC coefficient Coefficients!M20 = 0.0306114 = sqrt(rank/n_w), Post WFC 0.09183 nm.</t>
+          <t xml:space="preserve">white cells = inputs you edit; gray cells = formulas (computed) -- inputs: WFE columns C and G, Design WFE, WFE Requirement; the raw coefficient blocks on Coefficients (J:R) are tool-written values</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFS, HabEx reading (alpha = 1, the sigma passes whole): type 1 in Coefficients!M20; the payload re-rolls.</t>
+          <t xml:space="preserve">WFS: "WFS Sensing Error" (WFE row 20) sigma 3 nm is WHITE per-sample noise (Redding 2014 Eq. 32, the default ruled 2026-10-16): post-WFC coefficient Coefficients!M20 = 0.0306114 = sqrt(rank/n_w), Post WFC 0.09183 nm.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">budget e5hex1 from live sensitivities struct</t>
+          <t xml:space="preserve">WFS, HabEx reading (alpha = 1, the sigma passes whole): type 1 in Coefficients!M20; the payload re-rolls.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACOS_resources 85900c3</t>
+          <t xml:space="preserve">budget e5hex1 from live sensitivities struct</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MACOS_resources 1d10ab5</t>
         </is>
       </c>
     </row>

</xml_diff>